<commit_message>
feat(all): add Complexity Reason column to HigherEdu and Banking XLSX catalogues
- REASON_MAP covers all (complexity x pattern) combos for each domain
- HigherEdu: added Database Replication (CDC) and Batch (ETL) patterns
- Banking: added Batch (ETL) pattern
- All three catalogues now have 10-column J with derived rationale
</commit_message>
<xml_diff>
--- a/Banking/Catalogue/integration-details.xlsx
+++ b/Banking/Catalogue/integration-details.xlsx
@@ -21,18 +21,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collections &amp; Recovery" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer Onboarding &amp; Account M'!$A$1:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Payments &amp; Transfers'!$A$1:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lending &amp; Credit Management'!$A$1:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cards Management'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Deposits &amp; Savings Products'!$A$1:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Risk &amp; Compliance'!$A$1:$I$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Channels &amp; Digital Banking'!$A$1:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Finance, Treasury &amp; Settlement'!$A$1:$I$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Trade Finance'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Wealth Management'!$A$1:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Contact Center'!$A$1:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Collections &amp; Recovery'!$A$1:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer Onboarding &amp; Account M'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Payments &amp; Transfers'!$A$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Lending &amp; Credit Management'!$A$1:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cards Management'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Deposits &amp; Savings Products'!$A$1:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Risk &amp; Compliance'!$A$1:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Channels &amp; Digital Banking'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Finance, Treasury &amp; Settlement'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Trade Finance'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Wealth Management'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Contact Center'!$A$1:$J$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Collections &amp; Recovery'!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -477,6 +477,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +526,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -572,6 +578,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -619,6 +630,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -666,6 +682,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -713,6 +734,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -760,6 +786,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -807,6 +838,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -854,6 +890,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -901,6 +942,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -948,6 +994,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -995,6 +1046,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1042,6 +1098,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1089,6 +1150,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1136,6 +1202,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1183,6 +1254,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1230,6 +1306,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1277,6 +1358,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1324,6 +1410,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1371,9 +1462,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:J19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1384,7 +1480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1396,6 +1492,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1444,6 +1541,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1491,6 +1593,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1538,6 +1645,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1585,6 +1697,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1632,6 +1749,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1679,6 +1801,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1726,6 +1853,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1773,6 +1905,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1820,6 +1957,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1867,6 +2009,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1914,6 +2061,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1961,6 +2113,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2008,9 +2165,14 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2021,7 +2183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2033,6 +2195,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2081,6 +2244,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2128,6 +2296,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2175,6 +2348,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2222,6 +2400,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2269,6 +2452,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2316,6 +2504,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2363,6 +2556,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2410,6 +2608,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2457,6 +2660,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2504,6 +2712,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2551,6 +2764,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2598,6 +2816,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2645,6 +2868,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2692,9 +2920,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:J14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2705,7 +2938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2717,6 +2950,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2765,6 +2999,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2812,6 +3051,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2859,6 +3103,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2906,6 +3155,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2953,6 +3207,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3000,6 +3259,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3047,6 +3311,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3094,6 +3363,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Mission-critical event processing requiring guaranteed delivery, sequencing, and audit trail</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3141,6 +3415,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3188,6 +3467,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3235,6 +3519,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3282,6 +3571,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3329,6 +3623,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3376,6 +3675,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3423,9 +3727,14 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I15"/>
+  <autoFilter ref="A1:J15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3436,7 +3745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3448,6 +3757,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3496,6 +3806,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3543,6 +3858,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3590,6 +3910,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3637,6 +3962,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3684,6 +4014,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3731,6 +4066,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3778,6 +4118,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3825,6 +4170,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3872,6 +4222,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3919,6 +4274,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3966,6 +4326,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4013,6 +4378,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4060,6 +4430,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4107,6 +4482,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4154,6 +4534,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4201,6 +4586,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4248,6 +4638,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4295,6 +4690,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4342,6 +4742,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4389,6 +4794,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4436,6 +4846,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4483,6 +4898,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4530,6 +4950,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4577,9 +5002,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I24"/>
+  <autoFilter ref="A1:J24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4590,7 +5020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4602,6 +5032,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4650,6 +5081,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4697,6 +5133,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4744,6 +5185,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4791,6 +5237,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4838,6 +5289,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4885,6 +5341,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4932,6 +5393,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4979,6 +5445,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5026,6 +5497,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -5073,6 +5549,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5120,6 +5601,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Mission-critical event processing requiring guaranteed delivery, sequencing, and audit trail</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5167,6 +5653,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5214,6 +5705,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5261,6 +5757,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5308,6 +5809,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5355,6 +5861,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5402,6 +5913,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5449,6 +5965,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5496,6 +6017,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5543,6 +6069,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5590,6 +6121,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5637,6 +6173,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5684,6 +6225,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5731,9 +6277,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I24"/>
+  <autoFilter ref="A1:J24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5744,7 +6295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5756,6 +6307,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5804,6 +6356,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5851,6 +6408,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -5898,6 +6460,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5945,6 +6512,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -5992,6 +6564,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -6039,6 +6616,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6086,6 +6668,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -6133,6 +6720,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -6180,6 +6772,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -6227,6 +6824,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -6274,6 +6876,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6321,6 +6928,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6368,6 +6980,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -6415,6 +7032,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6462,6 +7084,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6509,6 +7136,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6556,6 +7188,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6603,6 +7240,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6650,6 +7292,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6697,6 +7344,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6744,6 +7396,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6791,6 +7448,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6838,6 +7500,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6885,6 +7552,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6932,6 +7604,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6979,9 +7656,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:J26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6992,7 +7674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7004,6 +7686,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7052,6 +7735,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -7099,6 +7787,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -7146,6 +7839,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -7193,6 +7891,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -7240,6 +7943,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -7287,6 +7995,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -7334,6 +8047,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -7381,6 +8099,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -7428,6 +8151,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -7475,6 +8203,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -7522,6 +8255,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -7569,6 +8307,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -7616,6 +8359,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -7663,6 +8411,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -7710,6 +8463,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -7757,6 +8515,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7804,6 +8567,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7851,6 +8619,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7898,6 +8671,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7945,6 +8723,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7992,6 +8775,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8039,9 +8827,14 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:J22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8052,7 +8845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8064,6 +8857,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8112,6 +8906,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -8159,6 +8958,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -8206,6 +9010,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -8253,6 +9062,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -8300,6 +9114,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -8347,6 +9166,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Straightforward periodic data transfer with no real-time constraints</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -8394,6 +9218,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -8441,6 +9270,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -8488,6 +9322,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -8535,6 +9374,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -8582,6 +9426,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -8629,6 +9478,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -8676,6 +9530,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate ETL process with data cleansing, enrichment, and staging requirements</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -8723,6 +9582,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate ETL process with data cleansing, enrichment, and staging requirements</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -8770,6 +9634,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -8817,6 +9686,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -8864,6 +9738,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate ETL process with data cleansing, enrichment, and staging requirements</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -8911,9 +9790,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I18"/>
+  <autoFilter ref="A1:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8924,7 +9808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8936,6 +9820,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8984,6 +9869,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -9031,6 +9921,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -9078,6 +9973,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9125,6 +10025,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9172,6 +10077,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9219,6 +10129,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -9266,6 +10181,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9313,6 +10233,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -9360,6 +10285,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9407,6 +10337,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9454,6 +10389,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9501,6 +10441,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9548,6 +10493,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9595,6 +10545,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -9642,6 +10597,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -9689,6 +10649,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -9736,6 +10701,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -9783,6 +10753,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -9830,9 +10805,14 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:J19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9843,7 +10823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9855,6 +10835,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9903,6 +10884,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -9950,6 +10936,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -9997,6 +10988,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate ETL process with data cleansing, enrichment, and staging requirements</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -10044,6 +11040,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -10091,6 +11092,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -10138,6 +11144,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -10185,6 +11196,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -10232,6 +11248,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -10279,6 +11300,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -10326,6 +11352,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -10373,6 +11404,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -10420,6 +11456,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -10467,6 +11508,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -10514,6 +11560,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Large-volume scheduled processing with data integrity validation and reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -10561,6 +11612,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -10608,6 +11664,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -10655,6 +11716,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -10702,6 +11768,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled batch transfer requiring field mapping, validation, and exception handling</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -10749,9 +11820,14 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:J19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10762,7 +11838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10774,6 +11850,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10822,6 +11899,11 @@
           <t>Complexity</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Complexity Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -10869,6 +11951,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -10916,6 +12003,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -10963,6 +12055,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -11010,6 +12107,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -11057,6 +12159,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -11104,6 +12211,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Simple event notification with fire-and-forget delivery semantics</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -11151,6 +12263,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -11198,6 +12315,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -11245,6 +12367,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -11292,6 +12419,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Real-time transaction boundary with strict consistency, auditing, and zero-data-loss requirements</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -11339,6 +12471,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Mission-critical event processing requiring guaranteed delivery, sequencing, and audit trail</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -11386,6 +12523,11 @@
           <t>Simple</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Direct API integration with minimal transformation and single-system lookup</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -11433,6 +12575,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -11480,6 +12627,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -11527,6 +12679,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>API integration requiring moderate transformation, error handling, and data reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -11574,9 +12731,14 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Event-driven integration with intermediate complexity in event routing and state management</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:J17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>